<commit_message>
Add named ranges and Apps Script API for the Dashboard
Adds 37 named ranges (KPI_* scalars + PM_Workload_Table) covering
every Dashboard metric, so a backend can address them by stable name
via the Sheets API instead of raw cell coordinates that break if the
layout changes. build_dashboard.py now asserts each row's label
before naming it, so a future layout edit fails loudly instead of
silently naming the wrong cell.

Also adds AppsScript/Code.gs: a doGet endpoint that serializes every
KPI_*/PM_Workload_Table named range to JSON, with an optional
API_TOKEN query-param check and a ?name= filter for single-value
polling. Setup steps are documented in the file's header comment.
</commit_message>
<xml_diff>
--- a/Property_Management_Tracker.xlsx
+++ b/Property_Management_Tracker.xlsx
@@ -20,6 +20,43 @@
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Lease Move Out Search'!$D$1:$K$1000</definedName>
     <definedName function="false" hidden="false" name="A11AC1" vbProcedure="false">#REF!</definedName>
+    <definedName function="false" hidden="false" name="KPI_ActiveUnits" vbProcedure="false">Dashboard!$C$10</definedName>
+    <definedName function="false" hidden="false" name="KPI_AncillaryIncome_Parking" vbProcedure="false">Dashboard!$C$41</definedName>
+    <definedName function="false" hidden="false" name="KPI_AncillaryIncome_PetFee" vbProcedure="false">Dashboard!$C$40</definedName>
+    <definedName function="false" hidden="false" name="KPI_AncillaryIncome_Storage" vbProcedure="false">Dashboard!$C$42</definedName>
+    <definedName function="false" hidden="false" name="KPI_GSTRate" vbProcedure="false">Dashboard!$C$5</definedName>
+    <definedName function="false" hidden="false" name="KPI_InvalidLeaseMoveIn_PMOnly" vbProcedure="false">Dashboard!$C$62</definedName>
+    <definedName function="false" hidden="false" name="KPI_InvalidMgmtAgreementDate_LeaseOnly" vbProcedure="false">Dashboard!$C$63</definedName>
+    <definedName function="false" hidden="false" name="KPI_InvalidMgmtAgreementDate_PMOnly" vbProcedure="false">Dashboard!$C$61</definedName>
+    <definedName function="false" hidden="false" name="KPI_LeasesExpiring30d" vbProcedure="false">Dashboard!$C$46</definedName>
+    <definedName function="false" hidden="false" name="KPI_LeasesExpiring60d" vbProcedure="false">Dashboard!$C$47</definedName>
+    <definedName function="false" hidden="false" name="KPI_LeasesExpiring90d" vbProcedure="false">Dashboard!$C$48</definedName>
+    <definedName function="false" hidden="false" name="KPI_LeasingFeeRevenue_ExclGST_PMOnly" vbProcedure="false">Dashboard!$C$35</definedName>
+    <definedName function="false" hidden="false" name="KPI_LeasingFeeRevenue_InclGST_LeaseOnly" vbProcedure="false">Dashboard!$C$36</definedName>
+    <definedName function="false" hidden="false" name="KPI_MgmtFeeRevenue_ExclGST" vbProcedure="false">Dashboard!$C$33</definedName>
+    <definedName function="false" hidden="false" name="KPI_MgmtFeeRevenue_InclGST_Est" vbProcedure="false">Dashboard!$C$34</definedName>
+    <definedName function="false" hidden="false" name="KPI_NewLeasesThisMonth" vbProcedure="false">Dashboard!$C$50</definedName>
+    <definedName function="false" hidden="false" name="KPI_NewOwnersThisMonth" vbProcedure="false">Dashboard!$C$54</definedName>
+    <definedName function="false" hidden="false" name="KPI_NewOwnersThisQuarter" vbProcedure="false">Dashboard!$C$55</definedName>
+    <definedName function="false" hidden="false" name="KPI_NewUnitsThisMonth" vbProcedure="false">Dashboard!$C$56</definedName>
+    <definedName function="false" hidden="false" name="KPI_NewUnitsThisQuarter" vbProcedure="false">Dashboard!$C$57</definedName>
+    <definedName function="false" hidden="false" name="KPI_OccupancyRate" vbProcedure="false">Dashboard!$C$15</definedName>
+    <definedName function="false" hidden="false" name="KPI_OccupiedMissingEmail" vbProcedure="false">Dashboard!$C$65</definedName>
+    <definedName function="false" hidden="false" name="KPI_OccupiedMissingPhone" vbProcedure="false">Dashboard!$C$66</definedName>
+    <definedName function="false" hidden="false" name="KPI_OccupiedMissingTenantName" vbProcedure="false">Dashboard!$C$64</definedName>
+    <definedName function="false" hidden="false" name="KPI_OccupiedUnits" vbProcedure="false">Dashboard!$C$12</definedName>
+    <definedName function="false" hidden="false" name="KPI_OwnerDisbursements_Combined" vbProcedure="false">Dashboard!$C$39</definedName>
+    <definedName function="false" hidden="false" name="KPI_OwnerDisbursements_LeaseOnly" vbProcedure="false">Dashboard!$C$38</definedName>
+    <definedName function="false" hidden="false" name="KPI_OwnerDisbursements_PMOnly" vbProcedure="false">Dashboard!$C$37</definedName>
+    <definedName function="false" hidden="false" name="KPI_RentRoll_LeaseOnly" vbProcedure="false">Dashboard!$C$32</definedName>
+    <definedName function="false" hidden="false" name="KPI_RentRoll_PMOnly" vbProcedure="false">Dashboard!$C$31</definedName>
+    <definedName function="false" hidden="false" name="KPI_ReportDate" vbProcedure="false">Dashboard!$C$4</definedName>
+    <definedName function="false" hidden="false" name="KPI_TakeOverUnits" vbProcedure="false">Dashboard!$C$14</definedName>
+    <definedName function="false" hidden="false" name="KPI_TerminatedUnits" vbProcedure="false">Dashboard!$C$11</definedName>
+    <definedName function="false" hidden="false" name="KPI_TotalUnits" vbProcedure="false">Dashboard!$C$9</definedName>
+    <definedName function="false" hidden="false" name="KPI_VacantActiveUnits" vbProcedure="false">Dashboard!$C$49</definedName>
+    <definedName function="false" hidden="false" name="KPI_VacantUnits" vbProcedure="false">Dashboard!$C$13</definedName>
+    <definedName function="false" hidden="false" name="PM_Workload_Table" vbProcedure="false">Dashboard!$B$18:$E$27</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>

</xml_diff>